<commit_message>
自动更新 周四 2026/06/25 16:32:59.65
</commit_message>
<xml_diff>
--- a/data/purchase_data.xlsx
+++ b/data/purchase_data.xlsx
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -143,8 +143,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,15 +512,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -556,7 +558,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>【Sheet 1: 使用说明】</t>
+          <t>【Sheet 1: 使用说明】当前页面 — 填写前请仔细阅读</t>
         </is>
       </c>
     </row>
@@ -566,7 +568,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>【Sheet 2: 采购数据（主表）】</t>
+          <t>【Sheet 2: 采购数据（主表）】在此表中填写实际采购数据</t>
         </is>
       </c>
     </row>
@@ -583,7 +585,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>📌 字段说明（共11列）：</t>
+          <t>📌 字段说明（共12列）：</t>
         </is>
       </c>
     </row>
@@ -895,20 +897,47 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>状态</t>
+          <t>满足状态</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
+          <t>是/否</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>是否满足需求：是/否/部分满足</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>采购状态</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
           <t>已到货</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>待审核/待发货/运输中/已到货/已取消</t>
         </is>
@@ -916,18 +945,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -939,13 +968,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
@@ -953,6 +982,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1008,7 +1038,12 @@
       </c>
       <c r="K1" s="8" t="inlineStr">
         <is>
-          <t>状态</t>
+          <t>满足状态</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>采购状态</t>
         </is>
       </c>
     </row>
@@ -1059,6 +1094,11 @@
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
           <t>已到货</t>
         </is>
       </c>
@@ -1106,6 +1146,11 @@
       <c r="J3" s="9" t="inlineStr"/>
       <c r="K3" s="9" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
           <t>运输中</t>
         </is>
       </c>
@@ -1153,6 +1198,11 @@
       <c r="J4" s="9" t="inlineStr"/>
       <c r="K4" s="9" t="inlineStr">
         <is>
+          <t>部分满足</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
           <t>待发货</t>
         </is>
       </c>
@@ -1199,6 +1249,11 @@
       </c>
       <c r="J5" s="9" t="inlineStr"/>
       <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>待审核</t>
         </is>
@@ -1216,6 +1271,7 @@
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr"/>
+      <c r="L6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr"/>
@@ -1229,6 +1285,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr"/>
@@ -1242,13 +1299,10 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>📝 填写说明：</t>
-        </is>
-      </c>
+      <c r="A9" s="10" t="inlineStr"/>
       <c r="B9" s="10" t="inlineStr"/>
       <c r="C9" s="10" t="inlineStr"/>
       <c r="D9" s="10" t="inlineStr"/>
@@ -1259,13 +1313,10 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr"/>
       <c r="K9" s="10" t="inlineStr"/>
+      <c r="L9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>• 请从第2行开始填写，不要修改第1行列名</t>
-        </is>
-      </c>
+      <c r="A10" s="10" t="inlineStr"/>
       <c r="B10" s="10" t="inlineStr"/>
       <c r="C10" s="10" t="inlineStr"/>
       <c r="D10" s="10" t="inlineStr"/>
@@ -1276,13 +1327,10 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>• 采购单号请保持唯一，不要重复</t>
-        </is>
-      </c>
+      <c r="A11" s="10" t="inlineStr"/>
       <c r="B11" s="10" t="inlineStr"/>
       <c r="C11" s="10" t="inlineStr"/>
       <c r="D11" s="10" t="inlineStr"/>
@@ -1293,13 +1341,10 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr"/>
       <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>• 总金额(CNY)可不填，上传后系统会自动计算</t>
-        </is>
-      </c>
+      <c r="A12" s="10" t="inlineStr"/>
       <c r="B12" s="10" t="inlineStr"/>
       <c r="C12" s="10" t="inlineStr"/>
       <c r="D12" s="10" t="inlineStr"/>
@@ -1310,13 +1355,10 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr"/>
       <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>• 日期格式固定为 YYYY-MM-DD（如 2025-06-01）</t>
-        </is>
-      </c>
+      <c r="A13" s="10" t="inlineStr"/>
       <c r="B13" s="10" t="inlineStr"/>
       <c r="C13" s="10" t="inlineStr"/>
       <c r="D13" s="10" t="inlineStr"/>
@@ -1327,13 +1369,10 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr"/>
       <c r="K13" s="10" t="inlineStr"/>
+      <c r="L13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>• 实际到货留空表示尚未到货</t>
-        </is>
-      </c>
+      <c r="A14" s="10" t="inlineStr"/>
       <c r="B14" s="10" t="inlineStr"/>
       <c r="C14" s="10" t="inlineStr"/>
       <c r="D14" s="10" t="inlineStr"/>
@@ -1344,8 +1383,277 @@
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="10" t="inlineStr"/>
       <c r="K14" s="10" t="inlineStr"/>
+      <c r="L14" s="10" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
+      <c r="E15" s="10" t="inlineStr"/>
+      <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="10" t="inlineStr"/>
+      <c r="I15" s="10" t="inlineStr"/>
+      <c r="J15" s="10" t="inlineStr"/>
+      <c r="K15" s="10" t="inlineStr"/>
+      <c r="L15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr"/>
+      <c r="E16" s="10" t="inlineStr"/>
+      <c r="F16" s="10" t="inlineStr"/>
+      <c r="G16" s="10" t="inlineStr"/>
+      <c r="H16" s="10" t="inlineStr"/>
+      <c r="I16" s="10" t="inlineStr"/>
+      <c r="J16" s="10" t="inlineStr"/>
+      <c r="K16" s="10" t="inlineStr"/>
+      <c r="L16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr"/>
+      <c r="C17" s="10" t="inlineStr"/>
+      <c r="D17" s="10" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr"/>
+      <c r="F17" s="10" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
+      <c r="I17" s="10" t="inlineStr"/>
+      <c r="J17" s="10" t="inlineStr"/>
+      <c r="K17" s="10" t="inlineStr"/>
+      <c r="L17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
+      <c r="F18" s="10" t="inlineStr"/>
+      <c r="G18" s="10" t="inlineStr"/>
+      <c r="H18" s="10" t="inlineStr"/>
+      <c r="I18" s="10" t="inlineStr"/>
+      <c r="J18" s="10" t="inlineStr"/>
+      <c r="K18" s="10" t="inlineStr"/>
+      <c r="L18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr"/>
+      <c r="B19" s="10" t="inlineStr"/>
+      <c r="C19" s="10" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr"/>
+      <c r="E19" s="10" t="inlineStr"/>
+      <c r="F19" s="10" t="inlineStr"/>
+      <c r="G19" s="10" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr"/>
+      <c r="I19" s="10" t="inlineStr"/>
+      <c r="J19" s="10" t="inlineStr"/>
+      <c r="K19" s="10" t="inlineStr"/>
+      <c r="L19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr"/>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr"/>
+      <c r="F20" s="10" t="inlineStr"/>
+      <c r="G20" s="10" t="inlineStr"/>
+      <c r="H20" s="10" t="inlineStr"/>
+      <c r="I20" s="10" t="inlineStr"/>
+      <c r="J20" s="10" t="inlineStr"/>
+      <c r="K20" s="10" t="inlineStr"/>
+      <c r="L20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="10" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr"/>
+      <c r="F21" s="10" t="inlineStr"/>
+      <c r="G21" s="10" t="inlineStr"/>
+      <c r="H21" s="10" t="inlineStr"/>
+      <c r="I21" s="10" t="inlineStr"/>
+      <c r="J21" s="10" t="inlineStr"/>
+      <c r="K21" s="10" t="inlineStr"/>
+      <c r="L21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr"/>
+      <c r="C22" s="10" t="inlineStr"/>
+      <c r="D22" s="10" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr"/>
+      <c r="F22" s="10" t="inlineStr"/>
+      <c r="G22" s="10" t="inlineStr"/>
+      <c r="H22" s="10" t="inlineStr"/>
+      <c r="I22" s="10" t="inlineStr"/>
+      <c r="J22" s="10" t="inlineStr"/>
+      <c r="K22" s="10" t="inlineStr"/>
+      <c r="L22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr"/>
+      <c r="C23" s="10" t="inlineStr"/>
+      <c r="D23" s="10" t="inlineStr"/>
+      <c r="E23" s="10" t="inlineStr"/>
+      <c r="F23" s="10" t="inlineStr"/>
+      <c r="G23" s="10" t="inlineStr"/>
+      <c r="H23" s="10" t="inlineStr"/>
+      <c r="I23" s="10" t="inlineStr"/>
+      <c r="J23" s="10" t="inlineStr"/>
+      <c r="K23" s="10" t="inlineStr"/>
+      <c r="L23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr"/>
+      <c r="B24" s="10" t="inlineStr"/>
+      <c r="C24" s="10" t="inlineStr"/>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr"/>
+      <c r="F24" s="10" t="inlineStr"/>
+      <c r="G24" s="10" t="inlineStr"/>
+      <c r="H24" s="10" t="inlineStr"/>
+      <c r="I24" s="10" t="inlineStr"/>
+      <c r="J24" s="10" t="inlineStr"/>
+      <c r="K24" s="10" t="inlineStr"/>
+      <c r="L24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr"/>
+      <c r="C25" s="10" t="inlineStr"/>
+      <c r="D25" s="10" t="inlineStr"/>
+      <c r="E25" s="10" t="inlineStr"/>
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="10" t="inlineStr"/>
+      <c r="J25" s="10" t="inlineStr"/>
+      <c r="K25" s="10" t="inlineStr"/>
+      <c r="L25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr"/>
+      <c r="B26" s="10" t="inlineStr"/>
+      <c r="C26" s="10" t="inlineStr"/>
+      <c r="D26" s="10" t="inlineStr"/>
+      <c r="E26" s="10" t="inlineStr"/>
+      <c r="F26" s="10" t="inlineStr"/>
+      <c r="G26" s="10" t="inlineStr"/>
+      <c r="H26" s="10" t="inlineStr"/>
+      <c r="I26" s="10" t="inlineStr"/>
+      <c r="J26" s="10" t="inlineStr"/>
+      <c r="K26" s="10" t="inlineStr"/>
+      <c r="L26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+      <c r="B27" s="10" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr"/>
+      <c r="F27" s="10" t="inlineStr"/>
+      <c r="G27" s="10" t="inlineStr"/>
+      <c r="H27" s="10" t="inlineStr"/>
+      <c r="I27" s="10" t="inlineStr"/>
+      <c r="J27" s="10" t="inlineStr"/>
+      <c r="K27" s="10" t="inlineStr"/>
+      <c r="L27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr"/>
+      <c r="B28" s="10" t="inlineStr"/>
+      <c r="C28" s="10" t="inlineStr"/>
+      <c r="D28" s="10" t="inlineStr"/>
+      <c r="E28" s="10" t="inlineStr"/>
+      <c r="F28" s="10" t="inlineStr"/>
+      <c r="G28" s="10" t="inlineStr"/>
+      <c r="H28" s="10" t="inlineStr"/>
+      <c r="I28" s="10" t="inlineStr"/>
+      <c r="J28" s="10" t="inlineStr"/>
+      <c r="K28" s="10" t="inlineStr"/>
+      <c r="L28" s="10" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr"/>
+      <c r="C29" s="10" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+      <c r="E29" s="10" t="inlineStr"/>
+      <c r="F29" s="10" t="inlineStr"/>
+      <c r="G29" s="10" t="inlineStr"/>
+      <c r="H29" s="10" t="inlineStr"/>
+      <c r="I29" s="10" t="inlineStr"/>
+      <c r="J29" s="10" t="inlineStr"/>
+      <c r="K29" s="10" t="inlineStr"/>
+      <c r="L29" s="10" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>📝 填写说明：</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>• 请从第2行开始填写，不要修改第1行列名</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>• 采购单号请保持唯一，不要重复</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>• 总金额(CNY)可不填，上传后系统会自动计算</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>• 日期格式固定为 YYYY-MM-DD（如 2025-06-01）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>• 实际到货列：未到货则留空</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>• 满足状态列：填写"是"/"否"/"部分满足"，用于计算满足率</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A33:L33"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="A32:L32"/>
+    <mergeCell ref="A36:L36"/>
+    <mergeCell ref="A31:L31"/>
+    <mergeCell ref="A34:L34"/>
+    <mergeCell ref="A35:L35"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
自动更新 周四 2026/06/25 16:52:32.89
</commit_message>
<xml_diff>
--- a/data/purchase_data.xlsx
+++ b/data/purchase_data.xlsx
@@ -897,12 +897,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>满足状态</t>
+          <t>满足率(%)</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>是/否</t>
+          <t>85.0</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>是否满足需求：是/否/部分满足</t>
+          <t>直接填写百分比数值，如 85、100、75.5、0</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="K1" s="8" t="inlineStr">
         <is>
-          <t>满足状态</t>
+          <t>满足率(%)</t>
         </is>
       </c>
       <c r="L1" s="8" t="inlineStr">
@@ -1092,10 +1092,8 @@
           <t>2025-06-14</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
+      <c r="K2" s="9" t="n">
+        <v>100</v>
       </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
@@ -1144,10 +1142,8 @@
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
+      <c r="K3" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
@@ -1196,10 +1192,8 @@
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr"/>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>部分满足</t>
-        </is>
+      <c r="K4" s="9" t="n">
+        <v>80</v>
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
@@ -1248,10 +1242,8 @@
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
+      <c r="K5" s="9" t="n">
+        <v>100</v>
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
@@ -1640,7 +1632,7 @@
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>• 满足状态列：填写"是"/"否"/"部分满足"，用于计算满足率</t>
+          <t>• 满足率(%)列：直接填写百分比数字，如 100、85、75.5、0</t>
         </is>
       </c>
     </row>

</xml_diff>